<commit_message>
Support page breaks in the study Excel import and update both templates
A section row of type 'فاصل صفحة' becomes a manual page break. The templates now list it, mark image alt text as required, fix the example rows that lacked alt text, and explain duplicate handling.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/blog_import_template.xlsx
+++ b/blog_import_template.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="72">
   <si>
     <t>استيراد المقالات بالجملة — دليل الاستخدام</t>
   </si>
@@ -63,10 +63,10 @@
     <t>نص  →  فقط اكتب النص مباشرة في خلية المحتوى (بدون "عنوان الحقل:"، النص وحده كافٍ).</t>
   </si>
   <si>
-    <t>صورة  →  رابط: ...  /  نص بديل: ...  /  تسمية: ... (نص بديل وتسمية اختياريان)</t>
-  </si>
-  <si>
-    <t>صورة+نص  →  رابط: ...  /  نص بديل: ...  /  الاتجاه: يمين أو يسار  /  النص: ...</t>
+    <t>صورة  →  رابط: ...  /  نص بديل: ... (إلزامي)  /  تسمية: ... (اختيارية)</t>
+  </si>
+  <si>
+    <t>صورة+نص  →  رابط: ...  /  نص بديل: ... (إلزامي)  /  الاتجاه: يمين أو يسار  /  النص: ...</t>
   </si>
   <si>
     <t>اقتباس  →  النص: ...  /  القائل: ... (القائل اختياري)</t>
@@ -103,6 +103,9 @@
   </si>
   <si>
     <t>• يمكنك رفع أكثر من ملف Excel في نفس العملية — إن فشل أحدها ستظهر النتيجة لكل ملف على حدة.</t>
+  </si>
+  <si>
+    <t>• النص البديل للصور إلزامي: القسم الذي يحتوي صورة بلا نص بديل لا يُستورد، وإذا كنت تُحدّث دراسة موجودة فلن يتغير أي شيء فيها.</t>
   </si>
   <si>
     <t>معرّف المقالة</t>
@@ -216,7 +219,8 @@
   <si>
     <t xml:space="preserve">رابط: https://example.com/images/writing-tips-section1.jpg
 الاتجاه: يمين
-النص: خصص وقتًا يوميًا ثابتًا للكتابة، حتى لو كان قصيرًا، فالانتظام أهم من الكمية.</t>
+النص: خصص وقتًا يوميًا ثابتًا للكتابة، حتى لو كان قصيرًا، فالانتظام أهم من الكمية.
+نص بديل: صورة توضيحية للنتائج</t>
   </si>
   <si>
     <t>وسوم</t>
@@ -685,7 +689,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A34"/>
+  <dimension ref="A1:A35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="105" customWidth="1"/>
@@ -861,9 +865,14 @@
         <v>29</v>
       </c>
     </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -888,86 +897,86 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B2" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>42</v>
-      </c>
       <c r="D2" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J2" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="K2" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="L2" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C3" s="7" t="s">
         <v>1</v>
@@ -976,19 +985,19 @@
         <v>1</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H3" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="I3" s="7" t="s">
         <v>49</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>48</v>
       </c>
       <c r="J3" s="7" t="s">
         <v>1</v>
@@ -1002,23 +1011,26 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="4">
+    <dataValidation type="list" allowBlank="1" sqref="G10:G500">
+      <formula1>"draft,published"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="G2:G500">
       <formula1>"draft,published"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="H2:H500">
+    <dataValidation type="list" allowBlank="1" sqref="H10:I500">
       <formula1>"نعم,لا"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="I2:I500">
+    <dataValidation type="list" allowBlank="1" sqref="H2:I500">
       <formula1>"نعم,لا"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1035,114 +1047,117 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" ht="45" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B2" s="7">
         <v>1</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" ht="45" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B3" s="7">
         <v>2</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" ht="45" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B4" s="7">
         <v>3</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" ht="45" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B5" s="7">
         <v>4</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B6" s="7">
         <v>1</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B7" s="7">
         <v>2</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation type="list" sqref="C10:C500">
+      <formula1>"نص,صورة,صورة+نص,اقتباس,PDF,صوت,فيديو,وسوم"</formula1>
+    </dataValidation>
     <dataValidation type="list" sqref="C2:C500">
       <formula1>"نص,صورة,صورة+نص,اقتباس,PDF,صوت,فيديو,وسوم"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>